<commit_message>
fixed joint torque plot test ok
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/trajectory_torque.xlsx
+++ b/dynamics/src/dynamics/xlsx/trajectory_torque.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>8.083067559448985e-07</v>
+        <v>-8.607942764446288e-07</v>
       </c>
       <c r="C2" t="n">
-        <v>-2.116247947839015</v>
+        <v>-2.116703292595321</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.5686659369108562</v>
+        <v>-0.5688644465987239</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2029582530255409</v>
+        <v>0.2029580551006954</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.007819211656537532</v>
+        <v>-0.007819146093197081</v>
       </c>
       <c r="G2" t="n">
-        <v>3.379912104099497e-13</v>
+        <v>6.373210404587942e-13</v>
       </c>
       <c r="H2" t="n">
-        <v>-3.725521159358323e-05</v>
+        <v>-5.024816524237395e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>1.570765263125453</v>
+        <v>1.570712727206166</v>
       </c>
       <c r="J2" t="n">
-        <v>6.352313794195675e-07</v>
+        <v>-5.596339013427496e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>5.354783488437533e-05</v>
+        <v>-6.321827447973192e-05</v>
       </c>
       <c r="L2" t="n">
-        <v>-5.52052983082831e-05</v>
+        <v>9.775921469554307e-05</v>
       </c>
       <c r="M2" t="n">
-        <v>8.262514472007753e-05</v>
+        <v>3.459211988374591e-05</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>1.24726346824483e-05</v>
+        <v>-1.328109993933822e-05</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -622,310 +622,695 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.634658397</v>
+        <v>0.634656412</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.006343995370715167</v>
+        <v>-0.006344255652562052</v>
       </c>
       <c r="C3" t="n">
-        <v>-4.391124171119079</v>
+        <v>-4.391480198566675</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.199940881285174</v>
+        <v>-1.200090903921308</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1927776680503781</v>
+        <v>0.1927643845310756</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.007460818206272883</v>
+        <v>-0.007460271315675355</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0002137797611873821</v>
+        <v>-0.0002137522227517451</v>
       </c>
       <c r="H3" t="n">
-        <v>-3.474327734050651e-05</v>
+        <v>-5.292290413959159e-05</v>
       </c>
       <c r="I3" t="n">
-        <v>1.221708421161667</v>
+        <v>1.221657443727283</v>
       </c>
       <c r="J3" t="n">
-        <v>-9.787280826518931e-06</v>
+        <v>-5.408258924467697e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>3.754703090008762e-05</v>
+        <v>-4.590195168016685e-05</v>
       </c>
       <c r="L3" t="n">
-        <v>-5.348891458060179e-05</v>
+        <v>8.029914448658627e-05</v>
       </c>
       <c r="M3" t="n">
-        <v>8.026561891246174e-05</v>
+        <v>3.395690090126462e-05</v>
       </c>
       <c r="N3" t="n">
-        <v>4.803531889725638e-06</v>
+        <v>-5.114880639859634e-06</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.6674958429530051</v>
+        <v>-0.6674954753767051</v>
       </c>
       <c r="P3" t="n">
-        <v>-1.993080419639126e-05</v>
+        <v>3.596639682341601e-06</v>
       </c>
       <c r="Q3" t="n">
-        <v>-3.059808277451274e-05</v>
+        <v>3.311385807907824e-05</v>
       </c>
       <c r="R3" t="n">
-        <v>3.282213282781939e-06</v>
+        <v>-3.338874503798576e-05</v>
       </c>
       <c r="S3" t="n">
-        <v>-4.512083645354445e-06</v>
+        <v>-1.214723904058337e-06</v>
       </c>
       <c r="T3" t="n">
-        <v>3.133836976475865e-06</v>
+        <v>-3.3369862814841e-06</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.4354760626788585</v>
+        <v>-0.4354790270034343</v>
       </c>
       <c r="V3" t="n">
-        <v>-1.300290964969919e-05</v>
+        <v>2.346474556197021e-06</v>
       </c>
       <c r="W3" t="n">
-        <v>-1.996227055619991e-05</v>
+        <v>2.160372800799666e-05</v>
       </c>
       <c r="X3" t="n">
-        <v>2.141324672427599e-06</v>
+        <v>-2.17830663103776e-05</v>
       </c>
       <c r="Y3" t="n">
-        <v>-2.94369536694622e-06</v>
+        <v>-7.924949356676907e-07</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1.079316795</v>
+        <v>1.079312824</v>
       </c>
       <c r="B4" t="n">
-        <v>0.01980238645787999</v>
+        <v>0.01980114544857106</v>
       </c>
       <c r="C4" t="n">
-        <v>-5.922659427724028</v>
+        <v>-5.922884934589324</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.608166578456327</v>
+        <v>-1.608257264866357</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1600232434414414</v>
+        <v>0.1600052375593384</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.006188053116851559</v>
+        <v>-0.006187332425029358</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.576586389114688e-13</v>
+        <v>-1.133186254362072e-12</v>
       </c>
       <c r="H4" t="n">
-        <v>-3.22313430874298e-05</v>
+        <v>-5.559764303680924e-05</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8726515791978807</v>
+        <v>0.8726021602484002</v>
       </c>
       <c r="J4" t="n">
-        <v>-2.020979303245743e-05</v>
+        <v>-5.220178835507896e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>2.15462269157999e-05</v>
+        <v>-2.858562888060179e-05</v>
       </c>
       <c r="L4" t="n">
-        <v>-5.177253085292049e-05</v>
+        <v>6.283907427762946e-05</v>
       </c>
       <c r="M4" t="n">
-        <v>7.790609310484596e-05</v>
+        <v>3.332168191878332e-05</v>
       </c>
       <c r="N4" t="n">
-        <v>5.649132609954101e-06</v>
+        <v>-6.015293661764254e-06</v>
       </c>
       <c r="O4" t="n">
         <v>-0.785</v>
       </c>
       <c r="P4" t="n">
-        <v>-2.343936888797773e-05</v>
+        <v>4.229784702352886e-06</v>
       </c>
       <c r="Q4" t="n">
-        <v>-3.598448624298561e-05</v>
+        <v>3.894315325119819e-05</v>
       </c>
       <c r="R4" t="n">
-        <v>3.860005203306146e-06</v>
+        <v>-3.926643074251094e-05</v>
       </c>
       <c r="S4" t="n">
-        <v>-5.306378607443421e-06</v>
+        <v>-1.428561390843358e-06</v>
       </c>
       <c r="T4" t="n">
-        <v>-9.524535600760555e-21</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>-2.285888544182533e-20</v>
+        <v>-3.428848125551243e-20</v>
       </c>
       <c r="W4" t="n">
-        <v>-1.523925696121689e-20</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>3.809814240304222e-21</v>
+        <v>9.143595001469983e-20</v>
       </c>
       <c r="Y4" t="n">
-        <v>-7.619628480608444e-21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.523975192</v>
+        <v>1.523969236</v>
       </c>
       <c r="B5" t="n">
-        <v>0.02424193837500446</v>
+        <v>0.02424077603161309</v>
       </c>
       <c r="C5" t="n">
-        <v>-6.853582702481053</v>
+        <v>-6.853666395103792</v>
       </c>
       <c r="D5" t="n">
-        <v>-1.861615736484003</v>
+        <v>-1.861647259753987</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1058327082731717</v>
+        <v>0.1058170167624434</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.004107655896773442</v>
+        <v>-0.004107045661611596</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.741827462713841e-13</v>
+        <v>-8.356289702164688e-13</v>
       </c>
       <c r="H5" t="n">
-        <v>-2.971940883435309e-05</v>
+        <v>-5.827238193402688e-05</v>
       </c>
       <c r="I5" t="n">
-        <v>0.523594737234095</v>
+        <v>0.5235468767695171</v>
       </c>
       <c r="J5" t="n">
-        <v>-3.063230523839593e-05</v>
+        <v>-5.032098746548097e-05</v>
       </c>
       <c r="K5" t="n">
-        <v>5.545422931512195e-06</v>
+        <v>-1.126930608103673e-05</v>
       </c>
       <c r="L5" t="n">
-        <v>-5.005614712523918e-05</v>
+        <v>4.537900406867267e-05</v>
       </c>
       <c r="M5" t="n">
-        <v>7.554656729723017e-05</v>
+        <v>3.268646293630203e-05</v>
       </c>
       <c r="N5" t="n">
-        <v>5.649132609954101e-06</v>
+        <v>-6.015293661764256e-06</v>
       </c>
       <c r="O5" t="n">
         <v>-0.785</v>
       </c>
       <c r="P5" t="n">
-        <v>-2.343936888797773e-05</v>
+        <v>4.22978470235288e-06</v>
       </c>
       <c r="Q5" t="n">
-        <v>-3.598448624298561e-05</v>
+        <v>3.894315325119821e-05</v>
       </c>
       <c r="R5" t="n">
-        <v>3.860005203306145e-06</v>
+        <v>-3.926643074251095e-05</v>
       </c>
       <c r="S5" t="n">
-        <v>-5.306378607443405e-06</v>
+        <v>-1.428561390843359e-06</v>
       </c>
       <c r="T5" t="n">
-        <v>7.619628480608443e-21</v>
+        <v>-1.142949375183748e-20</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>3.047851392243377e-20</v>
+        <v>7.619662501224988e-21</v>
       </c>
       <c r="W5" t="n">
-        <v>4.571777088365065e-20</v>
+        <v>9.143595001469985e-20</v>
       </c>
       <c r="X5" t="n">
-        <v>-7.619628480608443e-21</v>
+        <v>-1.219146000195998e-19</v>
       </c>
       <c r="Y5" t="n">
-        <v>8.000609904638864e-20</v>
+        <v>-2.381144531632809e-21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.96863359</v>
+        <v>1.968625648</v>
       </c>
       <c r="B6" t="n">
-        <v>0.02575747899224849</v>
+        <v>0.02575693952112269</v>
       </c>
       <c r="C6" t="n">
-        <v>-6.957892878539837</v>
+        <v>-6.957845170050613</v>
       </c>
       <c r="D6" t="n">
-        <v>-1.891387608582606</v>
+        <v>-1.891371397993239</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03949108853886829</v>
+        <v>0.03948288408350171</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.00155568008264346</v>
+        <v>-0.001555373398505579</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.773994933530165e-13</v>
+        <v>-5.062596348419481e-13</v>
       </c>
       <c r="H6" t="n">
-        <v>-2.720747458127638e-05</v>
+        <v>-6.094712083124452e-05</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1745378952703089</v>
+        <v>0.1744915932906341</v>
       </c>
       <c r="J6" t="n">
-        <v>-4.105481744433443e-05</v>
+        <v>-4.844018657588297e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>-1.045538105277552e-05</v>
+        <v>6.047016718528341e-06</v>
       </c>
       <c r="L6" t="n">
-        <v>-4.833976339755787e-05</v>
+        <v>2.791893385971586e-05</v>
       </c>
       <c r="M6" t="n">
-        <v>7.31870414896144e-05</v>
+        <v>3.205124395382074e-05</v>
       </c>
       <c r="N6" t="n">
-        <v>5.649132609954105e-06</v>
+        <v>-6.015293661764262e-06</v>
       </c>
       <c r="O6" t="n">
         <v>-0.785</v>
       </c>
       <c r="P6" t="n">
-        <v>-2.343936888797773e-05</v>
+        <v>4.229784702352887e-06</v>
       </c>
       <c r="Q6" t="n">
-        <v>-3.59844862429856e-05</v>
+        <v>3.89431532511982e-05</v>
       </c>
       <c r="R6" t="n">
-        <v>3.860005203306145e-06</v>
+        <v>-3.926643074251094e-05</v>
       </c>
       <c r="S6" t="n">
-        <v>-5.30637860744342e-06</v>
+        <v>-1.428561390843351e-06</v>
       </c>
       <c r="T6" t="n">
-        <v>7.619628480608443e-21</v>
+        <v>-1.523932500244997e-20</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.809814240304221e-20</v>
+        <v>2.095407187836871e-20</v>
       </c>
       <c r="W6" t="n">
-        <v>-1.523925696121689e-20</v>
+        <v>-1.219146000195998e-19</v>
       </c>
       <c r="X6" t="n">
-        <v>5.714721360456331e-21</v>
+        <v>1.523932500244997e-19</v>
       </c>
       <c r="Y6" t="n">
-        <v>-1.447729411315604e-19</v>
+        <v>3.857454141245149e-20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2.41328206</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.02416656039314061</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-6.222857369069071</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-1.693845573889676</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.03099766600911012</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.001159967420187153</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-1.619740826887431e-13</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-6.362185972846217e-05</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.1745636901882492</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-4.655938568628496e-05</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2.336333951809341e-05</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.045886365075906e-05</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3.141602497133945e-05</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-6.015293661764262e-06</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-0.785</v>
+      </c>
+      <c r="P7" t="n">
+        <v>4.229784702352887e-06</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3.894315325119819e-05</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-3.926643074251093e-05</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-1.428561390843351e-06</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1.523932500244997e-20</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-2.095407187836871e-20</v>
+      </c>
+      <c r="W7" t="n">
+        <v>6.095730000979988e-20</v>
+      </c>
+      <c r="X7" t="n">
+        <v>-1.219146000195998e-19</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>-3.857454141245149e-20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2.857938472</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.01966126977707582</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-4.737348668768861</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-1.292893497184308</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.09712510628393402</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.003711521731560527</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.779536741452479e-13</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-6.629659862567982e-05</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.5236189736671322</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-4.467858479668697e-05</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.067966231765846e-05</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-7.001206558197734e-06</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3.078080598885815e-05</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-6.015293661764259e-06</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-0.785</v>
+      </c>
+      <c r="P8" t="n">
+        <v>4.229784702352882e-06</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3.894315325119823e-05</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-3.926643074251098e-05</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-1.428561390843359e-06</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1.371539250220498e-19</v>
+      </c>
+      <c r="X8" t="n">
+        <v>-7.619662501224991e-20</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3.302594885</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.0127843786896672</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-2.680482902666805</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.7368733003255261</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-0.1509248682179561</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.005791585601252745</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.953549668607782e-13</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-6.897133752289746e-05</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.8726742571460151</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-4.279778390708897e-05</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5.799598511722354e-05</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-2.446127676715455e-05</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3.014558700637686e-05</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-6.015293661764259e-06</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-0.785</v>
+      </c>
+      <c r="P9" t="n">
+        <v>4.229784702352882e-06</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.894315325119823e-05</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-3.926643074251098e-05</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-1.428561390843359e-06</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>-1.371539250220498e-19</v>
+      </c>
+      <c r="X9" t="n">
+        <v>7.619662501224991e-20</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3.747251297</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.01478234630983929</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.1866136498034078</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.05055861715138786</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.1859859591552636</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.007174047719548699</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0002137522228702776</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-7.164607642011511e-05</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-1.221729540624898</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-4.091698301749097e-05</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7.53123079167886e-05</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-4.192134697611134e-05</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2.951036802389557e-05</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-5.114880639859635e-06</v>
+      </c>
+      <c r="O10" t="n">
+        <v>-0.6674954753767053</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3.596639682341598e-06</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.311385807907823e-05</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-3.338874503798574e-05</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-1.214723904058337e-06</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3.336986281484114e-06</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.4354790270034337</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-2.346474556196983e-06</v>
+      </c>
+      <c r="W10" t="n">
+        <v>-2.160372800799676e-05</v>
+      </c>
+      <c r="X10" t="n">
+        <v>2.178306631037765e-05</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>7.924949356676939e-07</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4.381907709</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.07128876404305597</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.568637031432717</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.7290843654787614</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.1976433587391635</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.00769914031863275</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0008507270885548451</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-7.432081531733275e-05</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-1.570784824103781</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-3.903618212789297e-05</v>
+      </c>
+      <c r="K11" t="n">
+        <v>9.262863071635365e-05</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-5.938141718506813e-05</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2.887514904141427e-05</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.328109993933819e-05</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1.73319276474404</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-9.338894576487968e-06</v>
+      </c>
+      <c r="W11" t="n">
+        <v>-8.598215471502544e-05</v>
+      </c>
+      <c r="X11" t="n">
+        <v>8.669591549075519e-05</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>3.154104798219605e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>